<commit_message>
I think I fix the random issue in classification part
</commit_message>
<xml_diff>
--- a/labeled/inspection/Hydrocare_ffinal.xlsx
+++ b/labeled/inspection/Hydrocare_ffinal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/inspection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C702EB-8383-5D45-BC65-A07EB911B6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA30EB7-91A0-5C4E-A6D9-8E13BB47E539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -534,7 +534,7 @@
   <dimension ref="A1:AC57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.5" customWidth="1"/>
     <col min="5" max="7" width="17.33203125" customWidth="1"/>
     <col min="8" max="8" width="33.33203125" customWidth="1"/>

</xml_diff>